<commit_message>
Memory map changed to overlay RAM
</commit_message>
<xml_diff>
--- a/memorymap.xlsx
+++ b/memorymap.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\OricScreenEditor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\xahmol\git\OricScreenEditorLOCI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2168A7-3277-4EA5-8C2C-B9FFE526DE27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F030A5-3B3F-41E0-AE91-6EFA87942C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38295" yWindow="240" windowWidth="28800" windowHeight="15345" xr2:uid="{FD51EA92-13D1-466E-83A2-BAF3E5CEB56D}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FD51EA92-13D1-466E-83A2-BAF3E5CEB56D}"/>
   </bookViews>
   <sheets>
     <sheet name="Memory map" sheetId="1" r:id="rId1"/>
-    <sheet name="Status bar design" sheetId="2" r:id="rId2"/>
+    <sheet name="Memory map old" sheetId="3" r:id="rId2"/>
+    <sheet name="Status bar design" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
   <si>
     <t>Memory map</t>
   </si>
@@ -159,14 +160,61 @@
   </si>
   <si>
     <t>AA00</t>
+  </si>
+  <si>
+    <t>Charset Std</t>
+  </si>
+  <si>
+    <t>Charset Alt</t>
+  </si>
+  <si>
+    <t>FFFF</t>
+  </si>
+  <si>
+    <t>Charset Swap</t>
+  </si>
+  <si>
+    <t>chars</t>
+  </si>
+  <si>
+    <t>lines of 40 chars</t>
+  </si>
+  <si>
+    <t>ORIC main RAM</t>
+  </si>
+  <si>
+    <t>RAM Area</t>
+  </si>
+  <si>
+    <t>ORIC overlay RAM</t>
+  </si>
+  <si>
+    <t>LOCI XRAM</t>
+  </si>
+  <si>
+    <t>Directory entries</t>
+  </si>
+  <si>
+    <t>Undo</t>
+  </si>
+  <si>
+    <t>9FFF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -194,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -204,6 +252,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -223,9 +275,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -263,7 +315,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -369,7 +421,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -511,7 +563,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -519,124 +571,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40711B7E-FB95-40EB-8A98-5CDE0B95CB31}">
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="1">
-        <v>500</v>
-      </c>
-      <c r="C3" s="1">
-        <f>+B4</f>
-        <v>9000</v>
-      </c>
-      <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D7" si="0">DEC2HEX(G3,4)</f>
-        <v>8B00</v>
-      </c>
-      <c r="E3" s="1">
-        <f t="shared" ref="E3:E7" si="1">HEX2DEC(B3)</f>
-        <v>1280</v>
-      </c>
-      <c r="F3" s="1">
-        <f t="shared" ref="F3" si="2">HEX2DEC(C3)</f>
-        <v>36864</v>
-      </c>
-      <c r="G3" s="1">
-        <f t="shared" ref="G3:G7" si="3">+F3-E3</f>
-        <v>35584</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="1">
-        <v>9000</v>
-      </c>
-      <c r="C4" s="1" t="str">
-        <f>+B5</f>
-        <v>AA00</v>
-      </c>
-      <c r="D4" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>1A00</v>
-      </c>
-      <c r="E4" s="1">
-        <f t="shared" si="1"/>
-        <v>36864</v>
-      </c>
-      <c r="F4" s="1">
-        <f t="shared" ref="F4" si="4">HEX2DEC(C4)</f>
-        <v>43520</v>
-      </c>
-      <c r="G4" s="1">
-        <f t="shared" si="3"/>
-        <v>6656</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="1" t="str">
-        <f>+B6</f>
-        <v>B100</v>
+      <c r="B5" s="1">
+        <v>400</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="D5" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>0700</v>
+        <f t="shared" ref="D5:D13" si="0">DEC2HEX(G5,4)</f>
+        <v>B000</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="1"/>
-        <v>43520</v>
+        <f t="shared" ref="E5:F11" si="1">HEX2DEC(B5)</f>
+        <v>1024</v>
       </c>
       <c r="F5" s="1">
-        <f t="shared" ref="F5:F6" si="5">HEX2DEC(C5)</f>
-        <v>45312</v>
+        <f t="shared" ref="F5" si="2">HEX2DEC(C5)</f>
+        <v>46080</v>
       </c>
       <c r="G5" s="1">
-        <f t="shared" si="3"/>
-        <v>1792</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <f t="shared" ref="G5:G7" si="3">+F5-E5</f>
+        <v>45056</v>
+      </c>
+      <c r="K5">
+        <f>+G5-'Memory map old'!G3</f>
+        <v>9472</v>
+      </c>
+      <c r="L5">
+        <f>+K5/1024</f>
+        <v>9.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>20</v>
@@ -653,7 +670,7 @@
         <v>45312</v>
       </c>
       <c r="F6" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>46080</v>
       </c>
       <c r="G6" s="1">
@@ -661,9 +678,9 @@
         <v>768</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -680,103 +697,242 @@
         <v>46336</v>
       </c>
       <c r="F7" s="1">
-        <f t="shared" ref="F7:F10" si="6">HEX2DEC(C7)</f>
+        <f t="shared" si="1"/>
         <v>47104</v>
       </c>
       <c r="G7" s="1">
         <f t="shared" si="3"/>
         <v>768</v>
       </c>
-      <c r="H7">
-        <f>+G7/8</f>
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1" t="str">
-        <f>+B9</f>
-        <v>BB80</v>
+        <f t="shared" ref="C6:C8" si="4">+B9</f>
+        <v>BFE0</v>
       </c>
       <c r="D8" s="1" t="str">
-        <f t="shared" ref="D8:D10" si="7">DEC2HEX(G8,4)</f>
-        <v>0280</v>
+        <f t="shared" si="0"/>
+        <v>0460</v>
       </c>
       <c r="E8" s="1">
-        <f t="shared" ref="E8:E10" si="8">HEX2DEC(B8)</f>
-        <v>47360</v>
+        <f t="shared" ref="E6:E9" si="5">HEX2DEC(B8)</f>
+        <v>48000</v>
       </c>
       <c r="F8" s="1">
-        <f t="shared" si="6"/>
-        <v>48000</v>
+        <f t="shared" ref="F6:F9" si="6">HEX2DEC(C8)</f>
+        <v>49120</v>
       </c>
       <c r="G8" s="1">
-        <f t="shared" ref="G8:G10" si="9">+F8-E8</f>
-        <v>640</v>
+        <f t="shared" ref="G6:G9" si="7">+F8-E8</f>
+        <v>1120</v>
       </c>
       <c r="H8">
-        <f>+G8/8</f>
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <f>+G8/40</f>
+        <v>28</v>
+      </c>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" s="1" t="str">
-        <f>+B10</f>
-        <v>BFE0</v>
+        <f>+B11</f>
+        <v>C000</v>
       </c>
       <c r="D9" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>0460</v>
+        <f t="shared" si="0"/>
+        <v>0020</v>
       </c>
       <c r="E9" s="1">
-        <f t="shared" si="8"/>
-        <v>48000</v>
+        <f t="shared" si="5"/>
+        <v>49120</v>
       </c>
       <c r="F9" s="1">
         <f t="shared" si="6"/>
-        <v>49120</v>
+        <v>49152</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" si="9"/>
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="1" t="s">
+        <f t="shared" si="7"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>0020</v>
-      </c>
-      <c r="E10" s="1">
-        <f t="shared" si="8"/>
-        <v>49120</v>
-      </c>
-      <c r="F10" s="1">
-        <f t="shared" si="6"/>
+      <c r="C11" s="1" t="str">
+        <f>DEC2HEX(F11,4)</f>
+        <v>F4FF</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="1"/>
         <v>49152</v>
       </c>
-      <c r="G10" s="1">
-        <f t="shared" si="9"/>
-        <v>32</v>
+      <c r="F11" s="1">
+        <f>+E12-1</f>
+        <v>62719</v>
+      </c>
+      <c r="G11" s="1">
+        <f>+F11-E11+1</f>
+        <v>13568</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <f>DEC2HEX(E12,4)</f>
+        <v>F500</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <f>DEC2HEX(F12,4)</f>
+        <v>FCFF</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f t="shared" ref="D12" si="8">DEC2HEX(G12,4)</f>
+        <v>0800</v>
+      </c>
+      <c r="E12" s="1">
+        <f>+F12-G12+1</f>
+        <v>62720</v>
+      </c>
+      <c r="F12" s="1">
+        <f>+E13-1</f>
+        <v>64767</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <f>DEC2HEX(E13,4)</f>
+        <v>FD00</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0300</v>
+      </c>
+      <c r="E13" s="1">
+        <f>+F13-G13+1</f>
+        <v>64768</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" ref="F13" si="9">HEX2DEC(C13)</f>
+        <v>65535</v>
+      </c>
+      <c r="G13" s="1">
+        <v>768</v>
+      </c>
+      <c r="H13">
+        <f>+G13/8</f>
+        <v>96</v>
+      </c>
+      <c r="I13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="1">
+        <v>8000</v>
+      </c>
+      <c r="C15" s="1" t="str">
+        <f>DEC2HEX(F15,4)</f>
+        <v>8BFF</v>
+      </c>
+      <c r="D15" s="1" t="str">
+        <f t="shared" ref="D15" si="10">DEC2HEX(G15,4)</f>
+        <v>0C00</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" ref="E15" si="11">HEX2DEC(B15)</f>
+        <v>32768</v>
+      </c>
+      <c r="F15" s="1">
+        <f>+E15+G15-1</f>
+        <v>35839</v>
+      </c>
+      <c r="G15" s="1">
+        <v>3072</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="1" t="str">
+        <f>DEC2HEX(E16,4)</f>
+        <v>8C00</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="1" t="str">
+        <f>DEC2HEX(G16,4)</f>
+        <v>1400</v>
+      </c>
+      <c r="E16">
+        <f>+F15+1</f>
+        <v>35840</v>
+      </c>
+      <c r="F16" s="1">
+        <f t="shared" ref="F16" si="12">HEX2DEC(C16)</f>
+        <v>40959</v>
+      </c>
+      <c r="G16">
+        <f>+F16-E16+1</f>
+        <v>5120</v>
       </c>
     </row>
   </sheetData>
@@ -786,14 +942,282 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26EB6BA1-A9D9-4906-8EE2-95549A5BEE7A}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1">
+        <v>500</v>
+      </c>
+      <c r="C3" s="1">
+        <f>+B4</f>
+        <v>9000</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <f t="shared" ref="D3:D10" si="0">DEC2HEX(G3,4)</f>
+        <v>8B00</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" ref="E3:F10" si="1">HEX2DEC(B3)</f>
+        <v>1280</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" si="1"/>
+        <v>36864</v>
+      </c>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G10" si="2">+F3-E3</f>
+        <v>35584</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1">
+        <v>9000</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <f>+B5</f>
+        <v>AA00</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>1A00</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="1"/>
+        <v>36864</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="1"/>
+        <v>43520</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="2"/>
+        <v>6656</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <f>+B6</f>
+        <v>B100</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0700</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="1"/>
+        <v>43520</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="1"/>
+        <v>45312</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="2"/>
+        <v>1792</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0300</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="1"/>
+        <v>45312</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="1"/>
+        <v>46080</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="2"/>
+        <v>768</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0300</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="1"/>
+        <v>46336</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="1"/>
+        <v>47104</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" si="2"/>
+        <v>768</v>
+      </c>
+      <c r="H7">
+        <f>+G7/8</f>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <f>+B9</f>
+        <v>BB80</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0280</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="1"/>
+        <v>47360</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="1"/>
+        <v>48000</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="2"/>
+        <v>640</v>
+      </c>
+      <c r="H8">
+        <f>+G8/8</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <f>+B10</f>
+        <v>BFE0</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0460</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="1"/>
+        <v>48000</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="1"/>
+        <v>49120</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="2"/>
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>0020</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="1"/>
+        <v>49120</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>49152</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="2"/>
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F65ED6-3220-425D-97D8-B8BB54836D97}">
   <dimension ref="A1:AN2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="40" width="5.7109375" style="2" customWidth="1"/>
+    <col min="1" max="40" width="5.7265625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A1" s="2">
         <v>0</v>
       </c>
@@ -915,7 +1339,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>

</xml_diff>